<commit_message>
Modified CAD files and add personalized 3d models for the PCB
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{876F6E9B-7ED2-4F00-9E75-8D13C9907CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B006F5-DC80-4451-82F3-61819308D3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -1038,8 +1038,8 @@
     <hyperlink ref="F14" r:id="rId12" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
     <hyperlink ref="F9" r:id="rId13" display="aa" xr:uid="{FABE7EDF-7DDE-462D-A255-256D487D3E16}"/>
     <hyperlink ref="F15" r:id="rId14" xr:uid="{26149171-8802-4F06-924C-935A7A889E39}"/>
-    <hyperlink ref="F16" r:id="rId15" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
-    <hyperlink ref="F17" r:id="rId16" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
+    <hyperlink ref="F17" r:id="rId15" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
+    <hyperlink ref="F16" r:id="rId16" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId17"/>

</xml_diff>

<commit_message>
Reorganized the repository and update README
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B006F5-DC80-4451-82F3-61819308D3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22F2B2C-058E-4331-91DA-4EC473C2D002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -162,7 +162,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +193,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -215,7 +222,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -223,6 +230,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -977,7 +985,7 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>14.65</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="5" t="s">
         <v>28</v>
       </c>
       <c r="G16">
@@ -1029,17 +1037,17 @@
     <hyperlink ref="F4" r:id="rId3" display="URL very long, shorted" xr:uid="{8E819B06-8183-48A6-B118-A91BE3A6E284}"/>
     <hyperlink ref="F5" r:id="rId4" display="URL very long, shorted" xr:uid="{1CE1FEDD-0883-422F-B918-52FF154AAD79}"/>
     <hyperlink ref="F6" r:id="rId5" display="URL very long, shorted" xr:uid="{ED55419D-2723-484E-911B-E97DC66A4B66}"/>
-    <hyperlink ref="F7" r:id="rId6" display="URL very long, shorted" xr:uid="{0DF8113F-FC99-4EE5-AA10-D3185C367D08}"/>
-    <hyperlink ref="F8" r:id="rId7" display="URL very long, shorted" xr:uid="{170C6CED-1834-4B92-A458-AE0F47B2B47E}"/>
-    <hyperlink ref="F10" r:id="rId8" display="URL very long, shorted" xr:uid="{38C32916-7239-4B3F-8936-54EC9D8E2A94}"/>
-    <hyperlink ref="F11" r:id="rId9" display="URL very long, shorted" xr:uid="{B869D917-0BBF-4FA2-9C08-6AB07DCF7FB0}"/>
-    <hyperlink ref="F12" r:id="rId10" display="URL very long, shorted" xr:uid="{6AF65191-9093-44CA-A434-65AC2B9E3853}"/>
-    <hyperlink ref="F13" r:id="rId11" display="URL very long, shorted" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
-    <hyperlink ref="F14" r:id="rId12" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
-    <hyperlink ref="F9" r:id="rId13" display="aa" xr:uid="{FABE7EDF-7DDE-462D-A255-256D487D3E16}"/>
-    <hyperlink ref="F15" r:id="rId14" xr:uid="{26149171-8802-4F06-924C-935A7A889E39}"/>
-    <hyperlink ref="F17" r:id="rId15" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
-    <hyperlink ref="F16" r:id="rId16" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
+    <hyperlink ref="F7" r:id="rId6" display="https://es.aliexpress.com/item/1005009122504274.html?spm=a2g0o.productlist.main.7.5f89748boATUNm&amp;algo_pvid=3013834c-bec4-4311-b0aa-2a86e15363f8&amp;algo_exp_id=3013834c-bec4-4311-b0aa-2a86e15363f8-6&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;107&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;fromPage&quot;%3A&quot;search&quot;%7D&amp;pdp_npi=6%40dis%21USD%212.94%212.94%21%21%212.94%212.94%21%402103212317704160897088421e55e9%2112000047991346899%21sea%21CL%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895&amp;curPageLogUid=i9Z3rLjRO4sc&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009122504274%7C_p_origin_prod%3A" xr:uid="{0DF8113F-FC99-4EE5-AA10-D3185C367D08}"/>
+    <hyperlink ref="F10" r:id="rId7" display="URL very long, shorted" xr:uid="{38C32916-7239-4B3F-8936-54EC9D8E2A94}"/>
+    <hyperlink ref="F11" r:id="rId8" display="URL very long, shorted" xr:uid="{B869D917-0BBF-4FA2-9C08-6AB07DCF7FB0}"/>
+    <hyperlink ref="F12" r:id="rId9" display="URL very long, shorted" xr:uid="{6AF65191-9093-44CA-A434-65AC2B9E3853}"/>
+    <hyperlink ref="F13" r:id="rId10" display="URL very long, shorted" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
+    <hyperlink ref="F14" r:id="rId11" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
+    <hyperlink ref="F9" r:id="rId12" display="aa" xr:uid="{FABE7EDF-7DDE-462D-A255-256D487D3E16}"/>
+    <hyperlink ref="F15" r:id="rId13" xr:uid="{26149171-8802-4F06-924C-935A7A889E39}"/>
+    <hyperlink ref="F17" r:id="rId14" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
+    <hyperlink ref="F16" r:id="rId15" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
+    <hyperlink ref="F8" r:id="rId16" display="URL very long, shorted" xr:uid="{170C6CED-1834-4B92-A458-AE0F47B2B47E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId17"/>

</xml_diff>

<commit_message>
Last details before summit
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22F2B2C-058E-4331-91DA-4EC473C2D002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934F9927-EC6C-4F21-957D-8D6B6D8B0468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t>Item</t>
   </si>
@@ -74,88 +74,112 @@
     <t>20pcs/lot nylon and tin-plated hinge board 12x24mm</t>
   </si>
   <si>
-    <t>Jumper Wires 120 pcs male-male female-male female-female</t>
-  </si>
-  <si>
     <t>LiPo Battery 3S 11.1V 2200mAh XT60</t>
   </si>
   <si>
     <t>IMAX B3 PRO 7.4V/11.1V 2S 3S 110-240V Compact Lipo Battery Balance Charger</t>
   </si>
   <si>
-    <t>Development board required for both control and air-to-ground communication</t>
-  </si>
-  <si>
-    <t>It allows for precise control with fewer pins for the servomotors used in the drone.</t>
-  </si>
-  <si>
-    <t>It allows bidirectional and real-time communication between the two ESP32s, enabling the sending of commands and the reading of sensors.</t>
-  </si>
-  <si>
-    <t>It delivers GPS data, speed, humidity, etc. Necessary for obtaining crucial data.</t>
-  </si>
-  <si>
-    <t>The voltage regulator, set to 3.3V, allows powering the variety of devices present.</t>
-  </si>
-  <si>
-    <t>Gyroscope, allows calculating aircraft attitude, acceleration, etc.</t>
-  </si>
-  <si>
-    <t>Medium torque and speed servomotors will allow the movement of the control surfaces</t>
-  </si>
-  <si>
-    <t>The brushless motor will be the heart of the drone and will provide thrust.</t>
-  </si>
-  <si>
-    <t>Propeller of suitable diameter to maximize the aircraft's maneuverability and speed</t>
-  </si>
-  <si>
-    <t>Nylon hinges will allow free movement of the control surfaces without compromising their integrity.</t>
-  </si>
-  <si>
-    <t>A charger for lithium polymer batteries is the safest way to charge this type of battery.</t>
-  </si>
-  <si>
     <t>ESP-32 Devkit 38 pins</t>
   </si>
   <si>
-    <t>8 pcs MG90S Servomotor</t>
-  </si>
-  <si>
     <t>Aliexpress</t>
   </si>
   <si>
     <t>Source</t>
   </si>
   <si>
-    <t>electric propeller APC 11X7</t>
-  </si>
-  <si>
     <t>NEEBRC 3542 1000KV  2-4S Outrunner Brushless Motor for RC Fixed Wing Airplane</t>
   </si>
   <si>
     <t>RC FPV Micro Camera AIO 5.8G 25MW 40CH 800TVL Transmitter LST-S4 + FPV Camera with OSD Parts for Racing Drone</t>
   </si>
   <si>
-    <t>The lithium polymer battery will provide sufficient voltage to operate the brushless motor.</t>
-  </si>
-  <si>
-    <t>RedHobby 70A  2-7S Brushless Electronic Speed ​​Controller ESC 5V BEC Output for RC Airplane</t>
-  </si>
-  <si>
-    <t>ESC and BEC that will allow to control the brushless motor and regulate the voltage to 5V</t>
-  </si>
-  <si>
-    <t>It will allow solderless testing and communication between differents parts of the plane</t>
-  </si>
-  <si>
     <t>RC832 Video Image Transmission Receiver, SKY 32S 5.8G FPV Wireless Upgrade</t>
   </si>
   <si>
-    <t>FPV Camera and transmisor that will allow to have video signal  in the plane</t>
-  </si>
-  <si>
-    <t>FPV Video receiver</t>
+    <t>4 pcs MG90S Servomotor</t>
+  </si>
+  <si>
+    <t>Lindinger</t>
+  </si>
+  <si>
+    <t>1/16"*3"*42" Balsa Sheet</t>
+  </si>
+  <si>
+    <t>1/4"*3"*24" Balsa Sheet</t>
+  </si>
+  <si>
+    <t>PCB</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>Balsa USA</t>
+  </si>
+  <si>
+    <t>1/8"*3"*24" Balsa Sheet</t>
+  </si>
+  <si>
+    <t>1/8"*1/8"*36" Balsa Strip</t>
+  </si>
+  <si>
+    <t>1/2"*1/2"*36" Balsa Strip</t>
+  </si>
+  <si>
+    <t>Dev board that will allow processing of telemetry, air-to-ground communication and autonomous operations based on vector operations</t>
+  </si>
+  <si>
+    <t>Servomotor driver that allows control of up to 16 servomotors using only 2 pins, mainly used to avoid using all the pins of the ESP32 and for more sophisticated control via binary control</t>
+  </si>
+  <si>
+    <t>Radio module that allows medium-range air-to-ground communication without major interference; a PLA antenna is added to maximize range.</t>
+  </si>
+  <si>
+    <t>GPS module that allows knowing the exact position of the aircraft along with its speed and altitude, key for both vector calculation and telemetry</t>
+  </si>
+  <si>
+    <t>The 3.3 Volt voltage regulator allows for the safe and continuous powering of sensitive modules such as the nrf24l01 directly from the VEC.</t>
+  </si>
+  <si>
+    <t>Magnetometer, gyroscope and accelerometer that will allow knowing the orientation and acceleration that the plane suffers in flight, also key for vector calculation thanks to being able to know the heading</t>
+  </si>
+  <si>
+    <t>Servomotors with metal gears that allow for high-performance and precise movement of control surfaces</t>
+  </si>
+  <si>
+    <t>A brushless motor that generates thrust for the aircraft was chosen in this case due to the aircraft's dimensions.It includes ESC and VEC which allows control via a microcontroller and voltage regulation from the LiPo battery.</t>
+  </si>
+  <si>
+    <t>AERONAUT CAM CARBON LIGHT 11/5 CLOCKWISE CW Popeller</t>
+  </si>
+  <si>
+    <t>Light carbon propeller designed to generate the maximum amount of thrust efficiently</t>
+  </si>
+  <si>
+    <t>Nylon hinges that allow free and controlled movement of the control surfaces</t>
+  </si>
+  <si>
+    <t>High-performance lithium polymer battery allowing sufficient voltage and current to be delivered to the motor thanks to its high discharge rate</t>
+  </si>
+  <si>
+    <t>The charger allows you to both balance and charge the LiPo battery safely.</t>
+  </si>
+  <si>
+    <t>AIO system for video recording and transmission, allows for a stable video signal</t>
+  </si>
+  <si>
+    <t>Video receiver to process the image and transform it into a USB signal for the application</t>
+  </si>
+  <si>
+    <t>Construction material, in this case mainly for the fuselage</t>
+  </si>
+  <si>
+    <t>Reinforcements for the control surfaces and fuselage</t>
+  </si>
+  <si>
+    <t>Circuit board to house all the electronics inside the aircraft</t>
   </si>
 </sst>
 </file>
@@ -250,8 +274,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G20" totalsRowShown="0">
-  <autoFilter ref="A1:G20" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G21" totalsRowShown="0">
+  <autoFilter ref="A1:G21" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B15320AC-39AF-49F6-85E9-A6118037BF1E}" name="Item"/>
     <tableColumn id="2" xr3:uid="{ED6149EA-8062-4364-85BB-6D993E2198BE}" name="Description"/>
@@ -261,7 +285,9 @@
       <calculatedColumnFormula>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{70DCF84D-F679-4074-84C0-742A0980B954}" name="Source"/>
-    <tableColumn id="7" xr3:uid="{74B24BCB-90B6-41C8-9F73-C54DA502394A}" name="Running Total ($ with Tax)"/>
+    <tableColumn id="7" xr3:uid="{74B24BCB-90B6-41C8-9F73-C54DA502394A}" name="Running Total ($ with Tax)">
+      <calculatedColumnFormula>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -584,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C67163-453F-4780-A8B8-99304635E2FD}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="98.21875" customWidth="1"/>
@@ -612,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -620,27 +646,27 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>4.83</v>
+        <v>4.2300000000000004</v>
       </c>
       <c r="E2">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>4.83</v>
+        <v>4.2300000000000004</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>5.75</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -648,24 +674,24 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>1.52</v>
+        <v>1.2</v>
       </c>
       <c r="E3">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>1.52</v>
+        <v>1.2</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G3">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>1.81</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -673,24 +699,24 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4">
-        <v>2.11</v>
+        <v>2.31</v>
       </c>
       <c r="E4">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>4.22</v>
+        <v>4.62</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G4">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>5.0199999999999996</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -698,24 +724,24 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>2.58</v>
+        <v>2.33</v>
       </c>
       <c r="E5">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>2.58</v>
+        <v>2.33</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G5">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>3.07</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -723,24 +749,24 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="E6">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G6">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -748,149 +774,149 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>2.14</v>
+        <v>2.31</v>
       </c>
       <c r="E7">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>2.14</v>
+        <v>2.31</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G7">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>2.5499999999999998</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8">
-        <v>13.21</v>
+        <v>7.26</v>
       </c>
       <c r="E8">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>13.21</v>
+        <v>14.52</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G8">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>15.72</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>15.5</v>
+        <v>39.520000000000003</v>
       </c>
       <c r="E9">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>15.5</v>
+        <v>39.520000000000003</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G9">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>18.45</v>
+        <v>47.03</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>6.9</v>
+      </c>
+      <c r="E10">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>6.9</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>8.2100000000000009</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>0.99</v>
+      </c>
+      <c r="E11">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>1.98</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>2.74</v>
-      </c>
-      <c r="E10">
-        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>2.74</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10">
-        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>3.26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="E11">
-        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11">
-        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>2.62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>0.99</v>
+        <v>19.57</v>
       </c>
       <c r="E12">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>0.99</v>
+        <v>19.57</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G12">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>1.18</v>
+        <v>23.29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -898,161 +924,256 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13">
-        <v>17.670000000000002</v>
+        <v>4.62</v>
       </c>
       <c r="E13">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>17.670000000000002</v>
+        <v>4.62</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G13">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>21.03</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14">
-        <v>7.36</v>
+        <v>14.65</v>
       </c>
       <c r="E14">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>7.36</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>28</v>
+        <v>14.65</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G14">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>8.76</v>
+        <v>17.43</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15">
-        <v>22.99</v>
+        <v>18.989999999999998</v>
       </c>
       <c r="E15">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>22.99</v>
+        <v>18.989999999999998</v>
       </c>
       <c r="F15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16">
+        <v>2.78</v>
+      </c>
+      <c r="E16">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>5.56</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="E17">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>4.0599999999999996</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>4.83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>3.16</v>
+      </c>
+      <c r="E18">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>3.16</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>28</v>
       </c>
-      <c r="G15">
-        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>27.36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16">
-        <v>14.65</v>
-      </c>
-      <c r="E16">
-        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>14.65</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G16">
-        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>17.43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
-        <v>18.989999999999998</v>
-      </c>
-      <c r="E17">
-        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>18.989999999999998</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G17">
-        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>22.6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="F18" s="3"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="F19" s="3"/>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>0.61</v>
+      </c>
+      <c r="E19">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>2.44</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>2.9</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="F20" s="3"/>
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20">
+        <v>2.46</v>
+      </c>
+      <c r="E20">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>4.92</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>5.85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>12.1</v>
+      </c>
+      <c r="E21">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>12.1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B30">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="URL very long, shorted" xr:uid="{99A62D6B-955A-465D-9C6A-2BAD046A9049}"/>
-    <hyperlink ref="F3" r:id="rId2" display="URL very long, shorted" xr:uid="{1B3F339E-6180-4794-AE9E-887FEDE8441C}"/>
-    <hyperlink ref="F4" r:id="rId3" display="URL very long, shorted" xr:uid="{8E819B06-8183-48A6-B118-A91BE3A6E284}"/>
-    <hyperlink ref="F5" r:id="rId4" display="URL very long, shorted" xr:uid="{1CE1FEDD-0883-422F-B918-52FF154AAD79}"/>
-    <hyperlink ref="F6" r:id="rId5" display="URL very long, shorted" xr:uid="{ED55419D-2723-484E-911B-E97DC66A4B66}"/>
-    <hyperlink ref="F7" r:id="rId6" display="https://es.aliexpress.com/item/1005009122504274.html?spm=a2g0o.productlist.main.7.5f89748boATUNm&amp;algo_pvid=3013834c-bec4-4311-b0aa-2a86e15363f8&amp;algo_exp_id=3013834c-bec4-4311-b0aa-2a86e15363f8-6&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;107&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;fromPage&quot;%3A&quot;search&quot;%7D&amp;pdp_npi=6%40dis%21USD%212.94%212.94%21%21%212.94%212.94%21%402103212317704160897088421e55e9%2112000047991346899%21sea%21CL%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895&amp;curPageLogUid=i9Z3rLjRO4sc&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009122504274%7C_p_origin_prod%3A" xr:uid="{0DF8113F-FC99-4EE5-AA10-D3185C367D08}"/>
-    <hyperlink ref="F10" r:id="rId7" display="URL very long, shorted" xr:uid="{38C32916-7239-4B3F-8936-54EC9D8E2A94}"/>
-    <hyperlink ref="F11" r:id="rId8" display="URL very long, shorted" xr:uid="{B869D917-0BBF-4FA2-9C08-6AB07DCF7FB0}"/>
-    <hyperlink ref="F12" r:id="rId9" display="URL very long, shorted" xr:uid="{6AF65191-9093-44CA-A434-65AC2B9E3853}"/>
-    <hyperlink ref="F13" r:id="rId10" display="URL very long, shorted" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
-    <hyperlink ref="F14" r:id="rId11" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
-    <hyperlink ref="F9" r:id="rId12" display="aa" xr:uid="{FABE7EDF-7DDE-462D-A255-256D487D3E16}"/>
-    <hyperlink ref="F15" r:id="rId13" xr:uid="{26149171-8802-4F06-924C-935A7A889E39}"/>
-    <hyperlink ref="F17" r:id="rId14" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
-    <hyperlink ref="F16" r:id="rId15" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
-    <hyperlink ref="F8" r:id="rId16" display="URL very long, shorted" xr:uid="{170C6CED-1834-4B92-A458-AE0F47B2B47E}"/>
+    <hyperlink ref="F4" r:id="rId2" display="URL very long, shorted" xr:uid="{8E819B06-8183-48A6-B118-A91BE3A6E284}"/>
+    <hyperlink ref="F5" r:id="rId3" display="URL very long, shorted" xr:uid="{1CE1FEDD-0883-422F-B918-52FF154AAD79}"/>
+    <hyperlink ref="F6" r:id="rId4" display="URL very long, shorted" xr:uid="{ED55419D-2723-484E-911B-E97DC66A4B66}"/>
+    <hyperlink ref="F7" r:id="rId5" display="https://es.aliexpress.com/item/1005009122504274.html?spm=a2g0o.productlist.main.7.5f89748boATUNm&amp;algo_pvid=3013834c-bec4-4311-b0aa-2a86e15363f8&amp;algo_exp_id=3013834c-bec4-4311-b0aa-2a86e15363f8-6&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;107&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;fromPage&quot;%3A&quot;search&quot;%7D&amp;pdp_npi=6%40dis%21USD%212.94%212.94%21%21%212.94%212.94%21%402103212317704160897088421e55e9%2112000047991346899%21sea%21CL%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895&amp;curPageLogUid=i9Z3rLjRO4sc&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009122504274%7C_p_origin_prod%3A" xr:uid="{0DF8113F-FC99-4EE5-AA10-D3185C367D08}"/>
+    <hyperlink ref="F11" r:id="rId6" display="URL very long, shorted" xr:uid="{6AF65191-9093-44CA-A434-65AC2B9E3853}"/>
+    <hyperlink ref="F12" r:id="rId7" display="URL very long, shorted" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
+    <hyperlink ref="F13" r:id="rId8" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
+    <hyperlink ref="F15" r:id="rId9" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
+    <hyperlink ref="F14" r:id="rId10" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
+    <hyperlink ref="F3" r:id="rId11" display="https://es.aliexpress.com/item/1005010790150348.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.3.101dnTiZnTiZhu&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40050.354490.0&amp;scm_id=1007.40050.354490.0&amp;scm-url=1007.40050.354490.0&amp;pvid=1402e862-8566-486e-90f8-f426f7e59b77&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40050.354490.0,pvid:1402e862-8566-486e-90f8-f426f7e59b77,tpp_buckets:668%232846%238116%232002&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;7&quot;%2C&quot;spu_best_type&quot;%3A&quot;price&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;sceneId&quot;%3A&quot;30050&quot;%2C&quot;fromPage&quot;%3A&quot;recommend&quot;%7D&amp;pdp_npi=6%40dis%21USD%218.09%211.20%21%21%2155.58%218.25%21%402101e07217707498748102094ee684%2112000053516946348%21rec%21CL%21%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895%3BpisId%3A5000000197836568&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A%7Cx_object_id%3A1005010790150348%7C_p_origin_prod%3A" xr:uid="{4C6DB327-3B29-497A-9836-280FC066EBB3}"/>
+    <hyperlink ref="F8" r:id="rId12" xr:uid="{92855497-DCF3-4FB4-954E-DA74E17A9E6E}"/>
+    <hyperlink ref="F9" r:id="rId13" xr:uid="{5E4566A1-A9A7-4ECD-96CD-A4912373900A}"/>
+    <hyperlink ref="F10" r:id="rId14" display="https://www.lindinger.at/en/AIRPLANES/ELECTRIC-POWERPLANTS/Propellers/Rigid-Propellers/AERONAUT-CAM-CARBON-LIGHT-11-5-CLOCKWISE-CW-Popeller/9709758" xr:uid="{78A19DBD-6F0A-4B57-ACE0-50E666B8B563}"/>
+    <hyperlink ref="F16" r:id="rId15" xr:uid="{9EA85452-3322-4931-8402-31752279EFDC}"/>
+    <hyperlink ref="F17" r:id="rId16" xr:uid="{34238490-F2E4-470E-BC83-EE055CABAEBD}"/>
+    <hyperlink ref="F18" r:id="rId17" xr:uid="{3E4D14A6-48CA-434C-A46C-C2589176B9AF}"/>
+    <hyperlink ref="F19" r:id="rId18" xr:uid="{D87BBA62-BFB9-4BA4-B0A1-BF2CCE34D658}"/>
+    <hyperlink ref="F20" r:id="rId19" xr:uid="{75546E6D-3F3A-4219-A15B-79C33E1B9949}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
   <tableParts count="1">
-    <tablePart r:id="rId18"/>
+    <tablePart r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Add M3 and M4 screws to the BOM and README, and create the initial CAD root file.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934F9927-EC6C-4F21-957D-8D6B6D8B0468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0BF822-7E93-4B75-B7C8-38C7C26BECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
   <si>
     <t>Item</t>
   </si>
@@ -180,6 +180,30 @@
   </si>
   <si>
     <t>Circuit board to house all the electronics inside the aircraft</t>
+  </si>
+  <si>
+    <t>M4x8 Screws</t>
+  </si>
+  <si>
+    <t>M3x8 Screws</t>
+  </si>
+  <si>
+    <t>M4x10 Screws</t>
+  </si>
+  <si>
+    <t>M4x6 Screws</t>
+  </si>
+  <si>
+    <t>M3x20 Screws</t>
+  </si>
+  <si>
+    <t>M4x12 Screws</t>
+  </si>
+  <si>
+    <t>Metric machine screws (M3/M4), zinc plated steel, for mechanical fastening and structural joining</t>
+  </si>
+  <si>
+    <t>Local Hardware Store</t>
   </si>
 </sst>
 </file>
@@ -274,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G21" totalsRowShown="0">
-  <autoFilter ref="A1:G21" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G27" totalsRowShown="0">
+  <autoFilter ref="A1:G27" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B15320AC-39AF-49F6-85E9-A6118037BF1E}" name="Item"/>
     <tableColumn id="2" xr3:uid="{ED6149EA-8062-4364-85BB-6D993E2198BE}" name="Description"/>
@@ -610,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C67163-453F-4780-A8B8-99304635E2FD}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="98.21875" customWidth="1"/>
@@ -1143,9 +1167,154 @@
         <v>12.1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B30">
-        <v>3</v>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>0.08</v>
+      </c>
+      <c r="E22">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.64</v>
+      </c>
+      <c r="F22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G22">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23">
+        <v>34</v>
+      </c>
+      <c r="D23">
+        <v>0.06</v>
+      </c>
+      <c r="E23">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>2.04</v>
+      </c>
+      <c r="F23" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>0.09</v>
+      </c>
+      <c r="E24">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.72</v>
+      </c>
+      <c r="F24" t="s">
+        <v>55</v>
+      </c>
+      <c r="G24">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25">
+        <v>0.08</v>
+      </c>
+      <c r="E25">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.32</v>
+      </c>
+      <c r="F25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G25">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26">
+        <v>0.1</v>
+      </c>
+      <c r="E26">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.4</v>
+      </c>
+      <c r="F26" t="s">
+        <v>55</v>
+      </c>
+      <c r="G26">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>0.1</v>
+      </c>
+      <c r="E27">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.8</v>
+      </c>
+      <c r="F27" t="s">
+        <v>55</v>
+      </c>
+      <c r="G27">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated BOM, PCB Files for include capacitors and connectors, added HUD Functions
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0BF822-7E93-4B75-B7C8-38C7C26BECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A51C43-1095-4CD7-B4C5-608501B1DFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
   <si>
     <t>Item</t>
   </si>
@@ -204,6 +204,60 @@
   </si>
   <si>
     <t>Local Hardware Store</t>
+  </si>
+  <si>
+    <t>XT60 Male conecctor</t>
+  </si>
+  <si>
+    <t>XT60 Female conector</t>
+  </si>
+  <si>
+    <t>JST Conector</t>
+  </si>
+  <si>
+    <t>40 pins socket pack</t>
+  </si>
+  <si>
+    <t>LiPo battery input connector, supplies power to the PCB main power rail.</t>
+  </si>
+  <si>
+    <t>High-current output connector, distributes power from the main rail to loads.</t>
+  </si>
+  <si>
+    <t>Low-current signal connector for auxiliary peripherals like the FPV camera.</t>
+  </si>
+  <si>
+    <t>High-frequency decoupling on the MPU9250 power supply line.</t>
+  </si>
+  <si>
+    <t>Local decoupling on the power supply lines of all modules.</t>
+  </si>
+  <si>
+    <t>Mid-frequency filtering on the PCA9685 and NEO-6M logic supply lines.</t>
+  </si>
+  <si>
+    <t>Voltage stabilization on the ESP32 and NRF24L01 power rails.</t>
+  </si>
+  <si>
+    <t>Interconnection headers for module mounting and replacement on the PCB.</t>
+  </si>
+  <si>
+    <t>Current spike absorption on the PCA9685 servo power rail.</t>
+  </si>
+  <si>
+    <t>Ceramic capacitor 10nf</t>
+  </si>
+  <si>
+    <t>Ceramic capacitor 100nf</t>
+  </si>
+  <si>
+    <t>Electrolitic capacitor 10uf</t>
+  </si>
+  <si>
+    <t>Electrolitic capacitor 100uf</t>
+  </si>
+  <si>
+    <t>Electrolitic capacitor 470uf</t>
   </si>
 </sst>
 </file>
@@ -298,8 +352,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G27" totalsRowShown="0">
-  <autoFilter ref="A1:G27" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}" name="Tabla1" displayName="Tabla1" ref="A1:G36" totalsRowShown="0">
+  <autoFilter ref="A1:G36" xr:uid="{11A09E66-F98C-436E-88B2-F7F65A97D7EA}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B15320AC-39AF-49F6-85E9-A6118037BF1E}" name="Item"/>
     <tableColumn id="2" xr3:uid="{ED6149EA-8062-4364-85BB-6D993E2198BE}" name="Description"/>
@@ -634,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C67163-453F-4780-A8B8-99304635E2FD}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="98.21875" customWidth="1"/>
@@ -1315,6 +1369,231 @@
       <c r="G27">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
         <v>0.95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>0.85</v>
+      </c>
+      <c r="E28">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.85</v>
+      </c>
+      <c r="F28" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <v>0.85</v>
+      </c>
+      <c r="E29">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.85</v>
+      </c>
+      <c r="F29" t="s">
+        <v>55</v>
+      </c>
+      <c r="G29">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>0.15</v>
+      </c>
+      <c r="E30">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.15</v>
+      </c>
+      <c r="F30" t="s">
+        <v>55</v>
+      </c>
+      <c r="G30">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
+      </c>
+      <c r="D31">
+        <v>0.6</v>
+      </c>
+      <c r="E31">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>1.2</v>
+      </c>
+      <c r="F31" t="s">
+        <v>55</v>
+      </c>
+      <c r="G31">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>0.08</v>
+      </c>
+      <c r="E32">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.08</v>
+      </c>
+      <c r="F32" t="s">
+        <v>55</v>
+      </c>
+      <c r="G32">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33">
+        <v>7</v>
+      </c>
+      <c r="D33">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E33">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.49000000000000005</v>
+      </c>
+      <c r="F33" t="s">
+        <v>55</v>
+      </c>
+      <c r="G33">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34">
+        <v>0.12</v>
+      </c>
+      <c r="E34">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.24</v>
+      </c>
+      <c r="F34" t="s">
+        <v>55</v>
+      </c>
+      <c r="G34">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>0.22</v>
+      </c>
+      <c r="E35">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.66</v>
+      </c>
+      <c r="F35" t="s">
+        <v>55</v>
+      </c>
+      <c r="G35">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E36">
+        <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F36" t="s">
+        <v>55</v>
+      </c>
+      <c r="G36">
+        <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
+        <v>0.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
build: generate PCB manufacturing files, update BOM, and package application releases
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cevac\XDF-001\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A51C43-1095-4CD7-B4C5-608501B1DFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BBD5B0-89AC-4519-B15D-B3A4073F251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57CB118E-8278-42F0-84AE-CA474A92FF74}"/>
   </bookViews>
@@ -98,9 +98,6 @@
     <t>RC832 Video Image Transmission Receiver, SKY 32S 5.8G FPV Wireless Upgrade</t>
   </si>
   <si>
-    <t>4 pcs MG90S Servomotor</t>
-  </si>
-  <si>
     <t>Lindinger</t>
   </si>
   <si>
@@ -116,9 +113,6 @@
     <t>JLCPCB</t>
   </si>
   <si>
-    <t>Balsa USA</t>
-  </si>
-  <si>
     <t>1/8"*3"*24" Balsa Sheet</t>
   </si>
   <si>
@@ -258,6 +252,12 @@
   </si>
   <si>
     <t>Electrolitic capacitor 470uf</t>
+  </si>
+  <si>
+    <t>Local Wood Store</t>
+  </si>
+  <si>
+    <t>8s MG90S Servomotor</t>
   </si>
 </sst>
 </file>
@@ -727,7 +727,7 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -752,7 +752,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -777,7 +777,7 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -802,7 +802,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -827,7 +827,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -852,7 +852,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -874,27 +874,27 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>7.26</v>
+        <v>16.66</v>
       </c>
       <c r="E8">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>14.52</v>
+        <v>16.66</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G8">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>17.28</v>
+        <v>19.829999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -902,7 +902,7 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -924,10 +924,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -940,7 +940,7 @@
         <v>6.9</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G10">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -952,7 +952,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -977,24 +977,24 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>19.57</v>
+        <v>10.54</v>
       </c>
       <c r="E12">
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
-        <v>19.57</v>
+        <v>10.54</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G12">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
-        <v>23.29</v>
+        <v>12.54</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1002,7 +1002,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1027,7 +1027,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1052,7 +1052,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1074,10 +1074,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -1089,8 +1089,8 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>5.56</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>26</v>
+      <c r="F16" t="s">
+        <v>72</v>
       </c>
       <c r="G16">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1099,10 +1099,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -1114,8 +1114,8 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>4.0599999999999996</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>26</v>
+      <c r="F17" t="s">
+        <v>72</v>
       </c>
       <c r="G17">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1124,10 +1124,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1139,8 +1139,8 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>3.16</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>26</v>
+      <c r="F18" t="s">
+        <v>72</v>
       </c>
       <c r="G18">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1149,10 +1149,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19">
         <v>4</v>
@@ -1164,8 +1164,8 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>2.44</v>
       </c>
-      <c r="F19" s="3" t="s">
-        <v>26</v>
+      <c r="F19" t="s">
+        <v>72</v>
       </c>
       <c r="G19">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1174,10 +1174,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -1189,8 +1189,8 @@
         <f>Tabla1[[#This Row],[Quantity ]]*Tabla1[[#This Row],[Unit price]]</f>
         <v>4.92</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>26</v>
+      <c r="F20" t="s">
+        <v>72</v>
       </c>
       <c r="G20">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1199,10 +1199,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1215,7 +1215,7 @@
         <v>12.1</v>
       </c>
       <c r="F21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G21">
         <v>12.1</v>
@@ -1223,10 +1223,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22">
         <v>8</v>
@@ -1239,7 +1239,7 @@
         <v>0.64</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G22">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1248,10 +1248,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23">
         <v>34</v>
@@ -1264,7 +1264,7 @@
         <v>2.04</v>
       </c>
       <c r="F23" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G23">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1273,10 +1273,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C24">
         <v>8</v>
@@ -1289,7 +1289,7 @@
         <v>0.72</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G24">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1298,10 +1298,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C25">
         <v>4</v>
@@ -1314,7 +1314,7 @@
         <v>0.32</v>
       </c>
       <c r="F25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G25">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1323,10 +1323,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
         <v>52</v>
-      </c>
-      <c r="B26" t="s">
-        <v>54</v>
       </c>
       <c r="C26">
         <v>4</v>
@@ -1339,7 +1339,7 @@
         <v>0.4</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G26">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C27">
         <v>8</v>
@@ -1364,7 +1364,7 @@
         <v>0.8</v>
       </c>
       <c r="F27" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G27">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1373,10 +1373,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1389,7 +1389,7 @@
         <v>0.85</v>
       </c>
       <c r="F28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G28">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1398,10 +1398,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1414,7 +1414,7 @@
         <v>0.85</v>
       </c>
       <c r="F29" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G29">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1423,10 +1423,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1439,7 +1439,7 @@
         <v>0.15</v>
       </c>
       <c r="F30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G30">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1448,10 +1448,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C31">
         <v>2</v>
@@ -1464,7 +1464,7 @@
         <v>1.2</v>
       </c>
       <c r="F31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G31">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1489,7 +1489,7 @@
         <v>0.08</v>
       </c>
       <c r="F32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G32">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1498,10 +1498,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C33">
         <v>7</v>
@@ -1514,7 +1514,7 @@
         <v>0.49000000000000005</v>
       </c>
       <c r="F33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G33">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1523,10 +1523,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -1539,7 +1539,7 @@
         <v>0.24</v>
       </c>
       <c r="F34" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G34">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1548,10 +1548,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C35">
         <v>3</v>
@@ -1564,7 +1564,7 @@
         <v>0.66</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G35">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1573,10 +1573,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -1589,7 +1589,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="F36" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G36">
         <f>ROUND(1.19*Tabla1[[#This Row],[Total Price]],2)</f>
@@ -1604,24 +1604,19 @@
     <hyperlink ref="F6" r:id="rId4" display="URL very long, shorted" xr:uid="{ED55419D-2723-484E-911B-E97DC66A4B66}"/>
     <hyperlink ref="F7" r:id="rId5" display="https://es.aliexpress.com/item/1005009122504274.html?spm=a2g0o.productlist.main.7.5f89748boATUNm&amp;algo_pvid=3013834c-bec4-4311-b0aa-2a86e15363f8&amp;algo_exp_id=3013834c-bec4-4311-b0aa-2a86e15363f8-6&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;107&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;fromPage&quot;%3A&quot;search&quot;%7D&amp;pdp_npi=6%40dis%21USD%212.94%212.94%21%21%212.94%212.94%21%402103212317704160897088421e55e9%2112000047991346899%21sea%21CL%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895&amp;curPageLogUid=i9Z3rLjRO4sc&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009122504274%7C_p_origin_prod%3A" xr:uid="{0DF8113F-FC99-4EE5-AA10-D3185C367D08}"/>
     <hyperlink ref="F11" r:id="rId6" display="URL very long, shorted" xr:uid="{6AF65191-9093-44CA-A434-65AC2B9E3853}"/>
-    <hyperlink ref="F12" r:id="rId7" display="URL very long, shorted" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
-    <hyperlink ref="F13" r:id="rId8" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
-    <hyperlink ref="F15" r:id="rId9" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
-    <hyperlink ref="F14" r:id="rId10" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
-    <hyperlink ref="F3" r:id="rId11" display="https://es.aliexpress.com/item/1005010790150348.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.3.101dnTiZnTiZhu&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40050.354490.0&amp;scm_id=1007.40050.354490.0&amp;scm-url=1007.40050.354490.0&amp;pvid=1402e862-8566-486e-90f8-f426f7e59b77&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40050.354490.0,pvid:1402e862-8566-486e-90f8-f426f7e59b77,tpp_buckets:668%232846%238116%232002&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;7&quot;%2C&quot;spu_best_type&quot;%3A&quot;price&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;sceneId&quot;%3A&quot;30050&quot;%2C&quot;fromPage&quot;%3A&quot;recommend&quot;%7D&amp;pdp_npi=6%40dis%21USD%218.09%211.20%21%21%2155.58%218.25%21%402101e07217707498748102094ee684%2112000053516946348%21rec%21CL%21%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895%3BpisId%3A5000000197836568&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A%7Cx_object_id%3A1005010790150348%7C_p_origin_prod%3A" xr:uid="{4C6DB327-3B29-497A-9836-280FC066EBB3}"/>
-    <hyperlink ref="F8" r:id="rId12" xr:uid="{92855497-DCF3-4FB4-954E-DA74E17A9E6E}"/>
-    <hyperlink ref="F9" r:id="rId13" xr:uid="{5E4566A1-A9A7-4ECD-96CD-A4912373900A}"/>
-    <hyperlink ref="F10" r:id="rId14" display="https://www.lindinger.at/en/AIRPLANES/ELECTRIC-POWERPLANTS/Propellers/Rigid-Propellers/AERONAUT-CAM-CARBON-LIGHT-11-5-CLOCKWISE-CW-Popeller/9709758" xr:uid="{78A19DBD-6F0A-4B57-ACE0-50E666B8B563}"/>
-    <hyperlink ref="F16" r:id="rId15" xr:uid="{9EA85452-3322-4931-8402-31752279EFDC}"/>
-    <hyperlink ref="F17" r:id="rId16" xr:uid="{34238490-F2E4-470E-BC83-EE055CABAEBD}"/>
-    <hyperlink ref="F18" r:id="rId17" xr:uid="{3E4D14A6-48CA-434C-A46C-C2589176B9AF}"/>
-    <hyperlink ref="F19" r:id="rId18" xr:uid="{D87BBA62-BFB9-4BA4-B0A1-BF2CCE34D658}"/>
-    <hyperlink ref="F20" r:id="rId19" xr:uid="{75546E6D-3F3A-4219-A15B-79C33E1B9949}"/>
+    <hyperlink ref="F13" r:id="rId7" display="URL very long, shorted" xr:uid="{E64F23B2-F270-4375-AA9A-287B3C507512}"/>
+    <hyperlink ref="F15" r:id="rId8" xr:uid="{D7B157C8-755D-460E-BB17-513ED15287F9}"/>
+    <hyperlink ref="F14" r:id="rId9" xr:uid="{4F798240-33D7-42F9-B6A3-5B5B9D2B205C}"/>
+    <hyperlink ref="F3" r:id="rId10" display="https://es.aliexpress.com/item/1005010790150348.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.3.101dnTiZnTiZhu&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40050.354490.0&amp;scm_id=1007.40050.354490.0&amp;scm-url=1007.40050.354490.0&amp;pvid=1402e862-8566-486e-90f8-f426f7e59b77&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40050.354490.0,pvid:1402e862-8566-486e-90f8-f426f7e59b77,tpp_buckets:668%232846%238116%232002&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;7&quot;%2C&quot;spu_best_type&quot;%3A&quot;price&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;sceneId&quot;%3A&quot;30050&quot;%2C&quot;fromPage&quot;%3A&quot;recommend&quot;%7D&amp;pdp_npi=6%40dis%21USD%218.09%211.20%21%21%2155.58%218.25%21%402101e07217707498748102094ee684%2112000053516946348%21rec%21CL%21%21ABX%211%210%21n_tag%3A-29910%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895%3BpisId%3A5000000197836568&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A%7Cx_object_id%3A1005010790150348%7C_p_origin_prod%3A" xr:uid="{4C6DB327-3B29-497A-9836-280FC066EBB3}"/>
+    <hyperlink ref="F8" r:id="rId11" display="https://es.aliexpress.com/item/1005007508741840.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.7.6ba16MtM6MtMrX&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40050.354490.0&amp;scm_id=1007.40050.354490.0&amp;scm-url=1007.40050.354490.0&amp;pvid=c06a098e-7118-4985-8ba4-cb29b0157d8b&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40050.354490.0,pvid:c06a098e-7118-4985-8ba4-cb29b0157d8b,tpp_buckets:668%232846%238111%231996&amp;pdp_ext_f=%7B&quot;order&quot;%3A&quot;259&quot;%2C&quot;eval&quot;%3A&quot;1&quot;%2C&quot;sceneId&quot;%3A&quot;30050&quot;%2C&quot;fromPage&quot;%3A&quot;recommend&quot;%7D&amp;pdp_npi=6%40dis%21USD%212.21%212.21%21%21%2115.20%2115.20%21%402101d97817747308544542936efa22%2112000041070118579%21rec%21CL%216626777930%21XZ%211%210%21n_tag%3A-29911%3Bd%3Aeb55f528%3Bm03_new_user%3A-29895&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A%7Cx_object_id%3A1005007508741840%7C_p_origin_prod%3A" xr:uid="{92855497-DCF3-4FB4-954E-DA74E17A9E6E}"/>
+    <hyperlink ref="F9" r:id="rId12" xr:uid="{5E4566A1-A9A7-4ECD-96CD-A4912373900A}"/>
+    <hyperlink ref="F10" r:id="rId13" display="https://www.lindinger.at/en/AIRPLANES/ELECTRIC-POWERPLANTS/Propellers/Rigid-Propellers/AERONAUT-CAM-CARBON-LIGHT-11-5-CLOCKWISE-CW-Popeller/9709758" xr:uid="{78A19DBD-6F0A-4B57-ACE0-50E666B8B563}"/>
+    <hyperlink ref="F12" r:id="rId14" display="https://es.aliexpress.com/item/1005007182410102.html" xr:uid="{480648C1-D138-4172-A1F3-6B9257B81573}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId20"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
   <tableParts count="1">
-    <tablePart r:id="rId21"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>